<commit_message>
Genericizar la plantilla para que sea reutilizable por cualquier empresa
Los datos de ejemplo del Sheet (docs/ERP_Sheet_Plantilla.xlsx) tenían
"Total Vet SAS" y un rubro veterinario (Concentrado Perro Adulto,
Distribuidora Mascotas, Veterinaria Amigo Fiel) heredados de cuando
usé al primer cliente real como referencia al construir la plantilla.
Ahora usan nombres neutros (Mi Empresa SAS, Línea/Producto/Proveedor/
Cliente Ejemplo) para no sesgar el ejemplo hacia un rubro específico.

También se quitan del repo los PDF/docx de la propuesta comercial de
Total Vet (no pertenecen a una plantilla genérica que se copia para
otros clientes) — quedan en disco pero fuera de git, vía .gitignore.

El código (React/Apps Script) ya no tenía ninguna referencia a Total
Vet, solo estos datos de ejemplo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ERP_Sheet_Plantilla.xlsx
+++ b/docs/ERP_Sheet_Plantilla.xlsx
@@ -787,12 +787,12 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Distribuidora Mascotas SAS</t>
+          <t>Proveedor Ejemplo SAS</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>3009876543</t>
+          <t>3000000001</t>
         </is>
       </c>
     </row>
@@ -1117,12 +1117,12 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Veterinaria Amigo Fiel</t>
+          <t>Cliente Ejemplo</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>3011112222</t>
+          <t>3000000002</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
@@ -1531,12 +1531,12 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Total Vet SAS</t>
+          <t>Mi Empresa SAS</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>900123456-7</t>
+          <t>900000000-0</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr"/>
@@ -1552,17 +1552,17 @@
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>Calle 10 # 5-20</t>
+          <t>Calle 1 # 2-34</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>3001234567</t>
+          <t>3000000000</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>contacto@totalvet.com</t>
+          <t>contacto@miempresa.com</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>admin@totalvet.com</t>
+          <t>admin@miempresa.com</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
@@ -2137,7 +2137,7 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Alimento para mascotas</t>
+          <t>Línea Ejemplo</t>
         </is>
       </c>
       <c r="C2" s="5" t="n">
@@ -2206,7 +2206,7 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Concentrado Perro Adulto 15kg</t>
+          <t>Producto Ejemplo</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">

</xml_diff>